<commit_message>
Added vertical tag to 2013 EM38 data
</commit_message>
<xml_diff>
--- a/Data/2014_F013B4_CO_ISOS/2014_F013B4_CO_ISOS_SoilAnalysis.xlsx
+++ b/Data/2014_F013B4_CO_ISOS/2014_F013B4_CO_ISOS_SoilAnalysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2014_F013B4_CO_ISOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B7C0AF-921C-4E6F-8854-0A2968FABC72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5501E6ED-F02F-4BB7-B48A-5982009108EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16320" yWindow="-28050" windowWidth="17910" windowHeight="25080" activeTab="3" xr2:uid="{8C00C1F2-89F9-4A44-A266-AB1BCF5C18BB}"/>
+    <workbookView xWindow="-1665" yWindow="-25290" windowWidth="27270" windowHeight="17295" xr2:uid="{8C00C1F2-89F9-4A44-A266-AB1BCF5C18BB}"/>
   </bookViews>
   <sheets>
     <sheet name="SoilDJH" sheetId="4" r:id="rId1"/>
@@ -446,9 +446,6 @@
     <t>Plot</t>
   </si>
   <si>
-    <t>2013d260EM38</t>
-  </si>
-  <si>
     <t>2015d118EM38</t>
   </si>
   <si>
@@ -1314,6 +1311,9 @@
   </si>
   <si>
     <t>2016-p0604</t>
+  </si>
+  <si>
+    <t>2013d260EM38V</t>
   </si>
 </sst>
 </file>
@@ -1696,13 +1696,13 @@
         <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E1" t="s">
         <v>134</v>
@@ -1713,7 +1713,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C2">
         <v>409014.13040000002</v>
@@ -1730,7 +1730,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C3">
         <v>409013.595399999</v>
@@ -1747,7 +1747,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C4">
         <v>409013.23430000001</v>
@@ -1764,7 +1764,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C5">
         <v>409012.73710000003</v>
@@ -1781,7 +1781,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C6">
         <v>409012.32490000001</v>
@@ -1798,7 +1798,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C7">
         <v>409011.88799999899</v>
@@ -1815,7 +1815,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C8">
         <v>408983.429999999</v>
@@ -1832,7 +1832,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C9">
         <v>408983.89409999899</v>
@@ -1849,7 +1849,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C10">
         <v>408984.30259999901</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C11">
         <v>408984.79070000001</v>
@@ -1883,7 +1883,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C12">
         <v>408985.21360000002</v>
@@ -1900,7 +1900,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C13">
         <v>408985.649299999</v>
@@ -1917,7 +1917,7 @@
         <v>131</v>
       </c>
       <c r="B14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C14">
         <v>408992.87400000001</v>
@@ -1934,7 +1934,7 @@
         <v>132</v>
       </c>
       <c r="B15" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C15">
         <v>408992.37520000001</v>
@@ -1951,7 +1951,7 @@
         <v>133</v>
       </c>
       <c r="B16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C16">
         <v>408991.93300000002</v>
@@ -1968,7 +1968,7 @@
         <v>134</v>
       </c>
       <c r="B17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C17">
         <v>408991.4412</v>
@@ -1985,7 +1985,7 @@
         <v>135</v>
       </c>
       <c r="B18" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C18">
         <v>408990.94170000002</v>
@@ -2002,7 +2002,7 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C19">
         <v>408957.18540000002</v>
@@ -2019,7 +2019,7 @@
         <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C20">
         <v>408956.76750000002</v>
@@ -2036,7 +2036,7 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C21">
         <v>408956.30570000003</v>
@@ -2053,7 +2053,7 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C22">
         <v>408955.91499999899</v>
@@ -2070,7 +2070,7 @@
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C23">
         <v>408955.44280000002</v>
@@ -2087,7 +2087,7 @@
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C24">
         <v>408955.01179999899</v>
@@ -2104,7 +2104,7 @@
         <v>136</v>
       </c>
       <c r="B25" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C25">
         <v>408962.41840000002</v>
@@ -2121,7 +2121,7 @@
         <v>137</v>
       </c>
       <c r="B26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C26">
         <v>408961.93680000002</v>
@@ -2138,7 +2138,7 @@
         <v>138</v>
       </c>
       <c r="B27" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C27">
         <v>408961.4645</v>
@@ -2155,7 +2155,7 @@
         <v>139</v>
       </c>
       <c r="B28" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C28">
         <v>408960.96830000001</v>
@@ -2172,7 +2172,7 @@
         <v>140</v>
       </c>
       <c r="B29" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C29">
         <v>408960.493599999</v>
@@ -2189,7 +2189,7 @@
         <v>19</v>
       </c>
       <c r="B30" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C30">
         <v>408926.557299999</v>
@@ -2206,7 +2206,7 @@
         <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C31">
         <v>408926.97979999898</v>
@@ -2223,7 +2223,7 @@
         <v>21</v>
       </c>
       <c r="B32" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C32">
         <v>408927.42930000002</v>
@@ -2240,7 +2240,7 @@
         <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C33">
         <v>408927.88109999901</v>
@@ -2257,7 +2257,7 @@
         <v>23</v>
       </c>
       <c r="B34" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C34">
         <v>408928.31640000001</v>
@@ -2274,7 +2274,7 @@
         <v>24</v>
       </c>
       <c r="B35" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C35">
         <v>408928.783999999</v>
@@ -2291,7 +2291,7 @@
         <v>141</v>
       </c>
       <c r="B36" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C36">
         <v>408936.025599999</v>
@@ -2308,7 +2308,7 @@
         <v>142</v>
       </c>
       <c r="B37" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C37">
         <v>408935.529199999</v>
@@ -2325,7 +2325,7 @@
         <v>143</v>
       </c>
       <c r="B38" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C38">
         <v>408935.03840000002</v>
@@ -2342,7 +2342,7 @@
         <v>144</v>
       </c>
       <c r="B39" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C39">
         <v>408934.55099999899</v>
@@ -2359,7 +2359,7 @@
         <v>145</v>
       </c>
       <c r="B40" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C40">
         <v>408934.06530000002</v>
@@ -2376,7 +2376,7 @@
         <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C41">
         <v>408901.33329999901</v>
@@ -2393,7 +2393,7 @@
         <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C42">
         <v>408900.9032</v>
@@ -2410,7 +2410,7 @@
         <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C43">
         <v>408900.44150000002</v>
@@ -2427,7 +2427,7 @@
         <v>28</v>
       </c>
       <c r="B44" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C44">
         <v>408899.99949999899</v>
@@ -2444,7 +2444,7 @@
         <v>29</v>
       </c>
       <c r="B45" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C45">
         <v>408899.580599999</v>
@@ -2461,7 +2461,7 @@
         <v>30</v>
       </c>
       <c r="B46" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C46">
         <v>408899.109999999</v>
@@ -2478,7 +2478,7 @@
         <v>146</v>
       </c>
       <c r="B47" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C47">
         <v>408906.29479999898</v>
@@ -2495,7 +2495,7 @@
         <v>147</v>
       </c>
       <c r="B48" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C48">
         <v>408905.79359999899</v>
@@ -2512,7 +2512,7 @@
         <v>148</v>
       </c>
       <c r="B49" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C49">
         <v>408905.32140000002</v>
@@ -2529,7 +2529,7 @@
         <v>149</v>
       </c>
       <c r="B50" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C50">
         <v>408904.8211</v>
@@ -2546,7 +2546,7 @@
         <v>150</v>
       </c>
       <c r="B51" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C51">
         <v>408904.35749999899</v>
@@ -2563,7 +2563,7 @@
         <v>31</v>
       </c>
       <c r="B52" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C52">
         <v>408870.67979999899</v>
@@ -2580,7 +2580,7 @@
         <v>32</v>
       </c>
       <c r="B53" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C53">
         <v>408871.13660000003</v>
@@ -2597,7 +2597,7 @@
         <v>33</v>
       </c>
       <c r="B54" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C54">
         <v>408871.57900000003</v>
@@ -2614,7 +2614,7 @@
         <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C55">
         <v>408872.00809999899</v>
@@ -2631,7 +2631,7 @@
         <v>35</v>
       </c>
       <c r="B56" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C56">
         <v>408872.451899999</v>
@@ -2648,7 +2648,7 @@
         <v>36</v>
       </c>
       <c r="B57" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C57">
         <v>408872.89059999899</v>
@@ -2665,7 +2665,7 @@
         <v>151</v>
       </c>
       <c r="B58" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C58">
         <v>408879.86940000003</v>
@@ -2682,7 +2682,7 @@
         <v>152</v>
       </c>
       <c r="B59" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C59">
         <v>408879.400499999</v>
@@ -2699,7 +2699,7 @@
         <v>153</v>
       </c>
       <c r="B60" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C60">
         <v>408878.89939999901</v>
@@ -2716,7 +2716,7 @@
         <v>154</v>
       </c>
       <c r="B61" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C61">
         <v>408878.41070000001</v>
@@ -2733,7 +2733,7 @@
         <v>155</v>
       </c>
       <c r="B62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C62">
         <v>408877.92340000003</v>
@@ -2750,7 +2750,7 @@
         <v>37</v>
       </c>
       <c r="B63" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C63">
         <v>408845.46089999902</v>
@@ -2767,7 +2767,7 @@
         <v>38</v>
       </c>
       <c r="B64" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C64">
         <v>408845.02049999899</v>
@@ -2784,7 +2784,7 @@
         <v>39</v>
       </c>
       <c r="B65" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C65">
         <v>408844.56319999899</v>
@@ -2801,7 +2801,7 @@
         <v>40</v>
       </c>
       <c r="B66" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C66">
         <v>408844.13500000001</v>
@@ -2818,7 +2818,7 @@
         <v>41</v>
       </c>
       <c r="B67" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C67">
         <v>408843.68329999998</v>
@@ -2835,7 +2835,7 @@
         <v>42</v>
       </c>
       <c r="B68" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C68">
         <v>408843.26179999899</v>
@@ -2852,7 +2852,7 @@
         <v>156</v>
       </c>
       <c r="B69" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C69">
         <v>408850.18070000003</v>
@@ -2869,7 +2869,7 @@
         <v>157</v>
       </c>
       <c r="B70" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C70">
         <v>408849.70020000002</v>
@@ -2886,7 +2886,7 @@
         <v>158</v>
       </c>
       <c r="B71" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C71">
         <v>408849.219199999</v>
@@ -2903,7 +2903,7 @@
         <v>159</v>
       </c>
       <c r="B72" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C72">
         <v>408848.73200000002</v>
@@ -2920,7 +2920,7 @@
         <v>160</v>
       </c>
       <c r="B73" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C73">
         <v>408848.231299999</v>
@@ -2937,7 +2937,7 @@
         <v>43</v>
       </c>
       <c r="B74" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C74">
         <v>408814.80080000003</v>
@@ -2954,7 +2954,7 @@
         <v>44</v>
       </c>
       <c r="B75" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C75">
         <v>408815.248499999</v>
@@ -2971,7 +2971,7 @@
         <v>45</v>
       </c>
       <c r="B76" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C76">
         <v>408815.666399999</v>
@@ -2988,7 +2988,7 @@
         <v>46</v>
       </c>
       <c r="B77" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C77">
         <v>408816.12689999898</v>
@@ -3005,7 +3005,7 @@
         <v>47</v>
       </c>
       <c r="B78" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C78">
         <v>408816.55469999899</v>
@@ -3022,7 +3022,7 @@
         <v>48</v>
       </c>
       <c r="B79" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C79">
         <v>408817.00829999999</v>
@@ -3039,7 +3039,7 @@
         <v>161</v>
       </c>
       <c r="B80" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C80">
         <v>408823.76260000002</v>
@@ -3056,7 +3056,7 @@
         <v>162</v>
       </c>
       <c r="B81" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C81">
         <v>408823.264399999</v>
@@ -3073,7 +3073,7 @@
         <v>163</v>
       </c>
       <c r="B82" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C82">
         <v>408822.77899999899</v>
@@ -3090,7 +3090,7 @@
         <v>164</v>
       </c>
       <c r="B83" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C83">
         <v>408822.312299999</v>
@@ -3107,7 +3107,7 @@
         <v>165</v>
       </c>
       <c r="B84" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C84">
         <v>408821.829399999</v>
@@ -3124,7 +3124,7 @@
         <v>49</v>
       </c>
       <c r="B85" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C85">
         <v>408788.581799999</v>
@@ -3141,7 +3141,7 @@
         <v>50</v>
       </c>
       <c r="B86" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C86">
         <v>408788.11670000001</v>
@@ -3158,7 +3158,7 @@
         <v>51</v>
       </c>
       <c r="B87" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C87">
         <v>408787.67560000002</v>
@@ -3175,7 +3175,7 @@
         <v>52</v>
       </c>
       <c r="B88" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C88">
         <v>408787.222799999</v>
@@ -3192,7 +3192,7 @@
         <v>53</v>
       </c>
       <c r="B89" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C89">
         <v>408786.80749999901</v>
@@ -3209,7 +3209,7 @@
         <v>54</v>
       </c>
       <c r="B90" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C90">
         <v>408786.36930000002</v>
@@ -3226,7 +3226,7 @@
         <v>166</v>
       </c>
       <c r="B91" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C91">
         <v>408793.35800000001</v>
@@ -3243,7 +3243,7 @@
         <v>167</v>
       </c>
       <c r="B92" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C92">
         <v>408792.866099999</v>
@@ -3260,7 +3260,7 @@
         <v>168</v>
       </c>
       <c r="B93" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C93">
         <v>408792.38530000002</v>
@@ -3277,7 +3277,7 @@
         <v>169</v>
       </c>
       <c r="B94" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C94">
         <v>408791.8947</v>
@@ -3294,7 +3294,7 @@
         <v>170</v>
       </c>
       <c r="B95" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C95">
         <v>408791.43050000002</v>
@@ -3311,7 +3311,7 @@
         <v>55</v>
       </c>
       <c r="B96" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C96">
         <v>408757.90980000002</v>
@@ -3328,7 +3328,7 @@
         <v>56</v>
       </c>
       <c r="B97" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C97">
         <v>408758.367499999</v>
@@ -3345,7 +3345,7 @@
         <v>57</v>
       </c>
       <c r="B98" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C98">
         <v>408758.807399999</v>
@@ -3362,7 +3362,7 @@
         <v>58</v>
       </c>
       <c r="B99" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C99">
         <v>408759.24219999899</v>
@@ -3379,7 +3379,7 @@
         <v>59</v>
       </c>
       <c r="B100" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C100">
         <v>408759.692099999</v>
@@ -3396,7 +3396,7 @@
         <v>60</v>
       </c>
       <c r="B101" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C101">
         <v>408760.11839999899</v>
@@ -3413,7 +3413,7 @@
         <v>171</v>
       </c>
       <c r="B102" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C102">
         <v>408766.92910000001</v>
@@ -3430,7 +3430,7 @@
         <v>172</v>
       </c>
       <c r="B103" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C103">
         <v>408766.46409999899</v>
@@ -3447,7 +3447,7 @@
         <v>173</v>
       </c>
       <c r="B104" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C104">
         <v>408765.99229999899</v>
@@ -3464,7 +3464,7 @@
         <v>174</v>
       </c>
       <c r="B105" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C105">
         <v>408765.47999999899</v>
@@ -3481,7 +3481,7 @@
         <v>175</v>
       </c>
       <c r="B106" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C106">
         <v>408765.01639999897</v>
@@ -3498,7 +3498,7 @@
         <v>61</v>
       </c>
       <c r="B107" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C107">
         <v>408674.80969999899</v>
@@ -3515,7 +3515,7 @@
         <v>62</v>
       </c>
       <c r="B108" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C108">
         <v>408674.3175</v>
@@ -3532,7 +3532,7 @@
         <v>63</v>
       </c>
       <c r="B109" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C109">
         <v>408673.885899999</v>
@@ -3549,7 +3549,7 @@
         <v>64</v>
       </c>
       <c r="B110" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C110">
         <v>408673.42570000002</v>
@@ -3566,7 +3566,7 @@
         <v>65</v>
       </c>
       <c r="B111" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C111">
         <v>408673.00859999901</v>
@@ -3583,7 +3583,7 @@
         <v>66</v>
       </c>
       <c r="B112" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C112">
         <v>408672.59139999899</v>
@@ -3600,7 +3600,7 @@
         <v>176</v>
       </c>
       <c r="B113" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C113">
         <v>408680.68900000001</v>
@@ -3617,7 +3617,7 @@
         <v>177</v>
       </c>
       <c r="B114" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C114">
         <v>408680.20289999899</v>
@@ -3634,7 +3634,7 @@
         <v>178</v>
       </c>
       <c r="B115" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C115">
         <v>408679.7047</v>
@@ -3651,7 +3651,7 @@
         <v>179</v>
       </c>
       <c r="B116" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C116">
         <v>408679.21340000001</v>
@@ -3668,7 +3668,7 @@
         <v>180</v>
       </c>
       <c r="B117" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C117">
         <v>408678.73639999999</v>
@@ -3698,13 +3698,13 @@
         <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E1" t="s">
         <v>134</v>
@@ -3715,7 +3715,7 @@
         <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C2">
         <v>409014.52750000003</v>
@@ -3732,7 +3732,7 @@
         <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C3">
         <v>409016.286599999</v>
@@ -3749,7 +3749,7 @@
         <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C4">
         <v>409015.53</v>
@@ -3766,7 +3766,7 @@
         <v>152</v>
       </c>
       <c r="B5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C5">
         <v>409014.96</v>
@@ -3783,7 +3783,7 @@
         <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C6">
         <v>409000.4903</v>
@@ -3800,7 +3800,7 @@
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C7">
         <v>408997.63040000002</v>
@@ -3817,7 +3817,7 @@
         <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C8">
         <v>408987.19380000001</v>
@@ -3834,7 +3834,7 @@
         <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C9">
         <v>408982.38959999901</v>
@@ -3851,7 +3851,7 @@
         <v>146</v>
       </c>
       <c r="B10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C10">
         <v>408985.71999999898</v>
@@ -3868,7 +3868,7 @@
         <v>147</v>
       </c>
       <c r="B11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C11">
         <v>408984.80999999901</v>
@@ -3885,7 +3885,7 @@
         <v>148</v>
       </c>
       <c r="B12" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C12">
         <v>408983.89</v>
@@ -3902,7 +3902,7 @@
         <v>149</v>
       </c>
       <c r="B13" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C13">
         <v>409002.11999999901</v>
@@ -3919,7 +3919,7 @@
         <v>150</v>
       </c>
       <c r="B14" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C14">
         <v>409003.26</v>
@@ -3936,7 +3936,7 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C15">
         <v>408957.29330000002</v>
@@ -3953,7 +3953,7 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C16">
         <v>408956.69130000001</v>
@@ -3970,7 +3970,7 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C17">
         <v>408956.084399999</v>
@@ -3987,7 +3987,7 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C18">
         <v>408955.49589999899</v>
@@ -4004,7 +4004,7 @@
         <v>74</v>
       </c>
       <c r="B19" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C19">
         <v>408973.7121</v>
@@ -4021,7 +4021,7 @@
         <v>75</v>
       </c>
       <c r="B20" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C20">
         <v>408968.074599999</v>
@@ -4038,7 +4038,7 @@
         <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C21">
         <v>408961.65999999898</v>
@@ -4055,7 +4055,7 @@
         <v>144</v>
       </c>
       <c r="B22" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C22">
         <v>408961.76</v>
@@ -4072,7 +4072,7 @@
         <v>145</v>
       </c>
       <c r="B23" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C23">
         <v>408963.02</v>
@@ -4089,7 +4089,7 @@
         <v>5</v>
       </c>
       <c r="B24" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C24">
         <v>408943.05879999901</v>
@@ -4106,7 +4106,7 @@
         <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C25">
         <v>408942.48519999901</v>
@@ -4123,7 +4123,7 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C26">
         <v>408941.846599999</v>
@@ -4140,7 +4140,7 @@
         <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C27">
         <v>408941.274299999</v>
@@ -4157,7 +4157,7 @@
         <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C28">
         <v>408928.85560000001</v>
@@ -4174,7 +4174,7 @@
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C29">
         <v>408928.25300000003</v>
@@ -4191,7 +4191,7 @@
         <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C30">
         <v>408927.64370000002</v>
@@ -4208,7 +4208,7 @@
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C31">
         <v>408927.035299999</v>
@@ -4225,7 +4225,7 @@
         <v>85</v>
       </c>
       <c r="B32" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C32">
         <v>408933.28</v>
@@ -4242,7 +4242,7 @@
         <v>140</v>
       </c>
       <c r="B33" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C33">
         <v>408933.33</v>
@@ -4259,7 +4259,7 @@
         <v>141</v>
       </c>
       <c r="B34" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C34">
         <v>408934.59</v>
@@ -4276,7 +4276,7 @@
         <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C35">
         <v>408914.35340000002</v>
@@ -4293,7 +4293,7 @@
         <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C36">
         <v>408913.7599</v>
@@ -4310,7 +4310,7 @@
         <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C37">
         <v>408913.14380000002</v>
@@ -4327,7 +4327,7 @@
         <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C38">
         <v>408912.52870000002</v>
@@ -4344,7 +4344,7 @@
         <v>86</v>
       </c>
       <c r="B39" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C39">
         <v>408904.549999999</v>
@@ -4361,7 +4361,7 @@
         <v>138</v>
       </c>
       <c r="B40" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C40">
         <v>408906.5</v>
@@ -4378,7 +4378,7 @@
         <v>139</v>
       </c>
       <c r="B41" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C41">
         <v>408905.239999999</v>
@@ -4395,7 +4395,7 @@
         <v>153</v>
       </c>
       <c r="B42" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C42">
         <v>408900.20380000002</v>
@@ -4412,7 +4412,7 @@
         <v>154</v>
       </c>
       <c r="B43" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C43">
         <v>408899.61949999898</v>
@@ -4429,7 +4429,7 @@
         <v>155</v>
       </c>
       <c r="B44" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C44">
         <v>408899.00260000001</v>
@@ -4446,7 +4446,7 @@
         <v>156</v>
       </c>
       <c r="B45" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C45">
         <v>408898.37829999899</v>
@@ -4463,7 +4463,7 @@
         <v>87</v>
       </c>
       <c r="B46" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C46">
         <v>408877.08</v>
@@ -4480,7 +4480,7 @@
         <v>134</v>
       </c>
       <c r="B47" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C47">
         <v>408879.09999999899</v>
@@ -4497,7 +4497,7 @@
         <v>135</v>
       </c>
       <c r="B48" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C48">
         <v>408877.859999999</v>
@@ -4514,7 +4514,7 @@
         <v>157</v>
       </c>
       <c r="B49" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C49">
         <v>408885.99040000001</v>
@@ -4531,7 +4531,7 @@
         <v>158</v>
       </c>
       <c r="B50" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C50">
         <v>408885.37439999898</v>
@@ -4548,7 +4548,7 @@
         <v>159</v>
       </c>
       <c r="B51" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C51">
         <v>408884.80279999902</v>
@@ -4565,7 +4565,7 @@
         <v>160</v>
       </c>
       <c r="B52" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C52">
         <v>408884.17149999901</v>
@@ -4582,7 +4582,7 @@
         <v>17</v>
       </c>
       <c r="B53" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C53">
         <v>408859.25290000002</v>
@@ -4599,7 +4599,7 @@
         <v>18</v>
       </c>
       <c r="B54" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C54">
         <v>408858.64659999899</v>
@@ -4616,7 +4616,7 @@
         <v>19</v>
       </c>
       <c r="B55" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C55">
         <v>408858.0344</v>
@@ -4633,7 +4633,7 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C56">
         <v>408857.44079999899</v>
@@ -4650,7 +4650,7 @@
         <v>21</v>
       </c>
       <c r="B57" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C57">
         <v>408845.03460000001</v>
@@ -4667,7 +4667,7 @@
         <v>22</v>
       </c>
       <c r="B58" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C58">
         <v>408844.4375</v>
@@ -4684,7 +4684,7 @@
         <v>23</v>
       </c>
       <c r="B59" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C59">
         <v>408843.829399999</v>
@@ -4701,7 +4701,7 @@
         <v>24</v>
       </c>
       <c r="B60" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C60">
         <v>408843.20490000001</v>
@@ -4718,7 +4718,7 @@
         <v>88</v>
       </c>
       <c r="B61" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C61">
         <v>408849.53</v>
@@ -4735,7 +4735,7 @@
         <v>132</v>
       </c>
       <c r="B62" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C62">
         <v>408849.489999999</v>
@@ -4752,7 +4752,7 @@
         <v>133</v>
       </c>
       <c r="B63" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C63">
         <v>408850.72999999899</v>
@@ -4769,7 +4769,7 @@
         <v>25</v>
       </c>
       <c r="B64" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C64">
         <v>408830.81489999901</v>
@@ -4786,7 +4786,7 @@
         <v>26</v>
       </c>
       <c r="B65" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C65">
         <v>408830.206899999</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="B66" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C66">
         <v>408829.59519999899</v>
@@ -4820,7 +4820,7 @@
         <v>28</v>
       </c>
       <c r="B67" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C67">
         <v>408828.99920000002</v>
@@ -4837,7 +4837,7 @@
         <v>29</v>
       </c>
       <c r="B68" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C68">
         <v>408816.59179999901</v>
@@ -4854,7 +4854,7 @@
         <v>30</v>
       </c>
       <c r="B69" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C69">
         <v>408815.986199999</v>
@@ -4871,7 +4871,7 @@
         <v>31</v>
       </c>
       <c r="B70" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C70">
         <v>408815.39</v>
@@ -4888,7 +4888,7 @@
         <v>32</v>
       </c>
       <c r="B71" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C71">
         <v>408814.777</v>
@@ -4905,7 +4905,7 @@
         <v>89</v>
       </c>
       <c r="B72" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C72">
         <v>408821.01</v>
@@ -4922,7 +4922,7 @@
         <v>128</v>
       </c>
       <c r="B73" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C73">
         <v>408821.109999999</v>
@@ -4939,7 +4939,7 @@
         <v>129</v>
       </c>
       <c r="B74" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C74">
         <v>408822.35</v>
@@ -4956,7 +4956,7 @@
         <v>33</v>
       </c>
       <c r="B75" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C75">
         <v>408802.449499999</v>
@@ -4973,7 +4973,7 @@
         <v>34</v>
       </c>
       <c r="B76" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C76">
         <v>408801.83819999901</v>
@@ -4990,7 +4990,7 @@
         <v>35</v>
       </c>
       <c r="B77" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C77">
         <v>408801.21379999898</v>
@@ -5007,7 +5007,7 @@
         <v>36</v>
       </c>
       <c r="B78" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C78">
         <v>408800.62819999899</v>
@@ -5024,7 +5024,7 @@
         <v>37</v>
       </c>
       <c r="B79" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C79">
         <v>408788.22350000002</v>
@@ -5041,7 +5041,7 @@
         <v>38</v>
       </c>
       <c r="B80" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C80">
         <v>408787.60700000002</v>
@@ -5058,7 +5058,7 @@
         <v>39</v>
       </c>
       <c r="B81" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C81">
         <v>408787.00040000002</v>
@@ -5075,7 +5075,7 @@
         <v>40</v>
       </c>
       <c r="B82" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C82">
         <v>408786.40159999899</v>
@@ -5092,7 +5092,7 @@
         <v>90</v>
       </c>
       <c r="B83" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C83">
         <v>408792.64</v>
@@ -5109,7 +5109,7 @@
         <v>126</v>
       </c>
       <c r="B84" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C84">
         <v>408794.59</v>
@@ -5126,7 +5126,7 @@
         <v>127</v>
       </c>
       <c r="B85" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C85">
         <v>408793.34999999899</v>
@@ -5143,7 +5143,7 @@
         <v>41</v>
       </c>
       <c r="B86" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C86">
         <v>408773.99790000002</v>
@@ -5160,7 +5160,7 @@
         <v>42</v>
       </c>
       <c r="B87" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C87">
         <v>408773.39649999898</v>
@@ -5177,7 +5177,7 @@
         <v>43</v>
       </c>
       <c r="B88" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C88">
         <v>408772.784099999</v>
@@ -5194,7 +5194,7 @@
         <v>44</v>
       </c>
       <c r="B89" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C89">
         <v>408772.17050000001</v>
@@ -5211,7 +5211,7 @@
         <v>45</v>
       </c>
       <c r="B90" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C90">
         <v>408759.7758</v>
@@ -5228,7 +5228,7 @@
         <v>46</v>
       </c>
       <c r="B91" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C91">
         <v>408759.1692</v>
@@ -5245,7 +5245,7 @@
         <v>47</v>
       </c>
       <c r="B92" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C92">
         <v>408758.57179999899</v>
@@ -5262,7 +5262,7 @@
         <v>48</v>
       </c>
       <c r="B93" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C93">
         <v>408757.959299999</v>
@@ -5279,7 +5279,7 @@
         <v>91</v>
       </c>
       <c r="B94" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C94">
         <v>408764.2</v>
@@ -5296,7 +5296,7 @@
         <v>122</v>
       </c>
       <c r="B95" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C95">
         <v>408766.09</v>
@@ -5313,7 +5313,7 @@
         <v>123</v>
       </c>
       <c r="B96" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C96">
         <v>408764.84999999899</v>
@@ -5330,7 +5330,7 @@
         <v>67</v>
       </c>
       <c r="B97" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C97">
         <v>408685.49530000001</v>
@@ -5347,7 +5347,7 @@
         <v>68</v>
       </c>
       <c r="B98" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C98">
         <v>408676.1875</v>
@@ -5364,7 +5364,7 @@
         <v>70</v>
       </c>
       <c r="B99" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C99">
         <v>408673.02689999901</v>
@@ -5381,7 +5381,7 @@
         <v>94</v>
       </c>
       <c r="B100" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C100">
         <v>408678.94</v>
@@ -5398,7 +5398,7 @@
         <v>113</v>
       </c>
       <c r="B101" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C101">
         <v>408680.549999999</v>
@@ -5415,7 +5415,7 @@
         <v>114</v>
       </c>
       <c r="B102" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C102">
         <v>408679.679999999</v>
@@ -5432,7 +5432,7 @@
         <v>115</v>
       </c>
       <c r="B103" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C103">
         <v>408678.72999999899</v>
@@ -5462,211 +5462,211 @@
         <v>121</v>
       </c>
       <c r="C1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>137</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>139</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>140</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>141</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>142</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>143</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>144</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>145</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>146</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>147</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>148</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>149</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>150</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>151</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>152</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>153</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>154</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>155</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>156</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>157</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>158</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>159</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>160</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>161</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>162</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>163</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>164</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>165</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>166</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>167</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>168</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>169</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>170</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>171</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>172</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>173</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>174</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>175</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>176</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>177</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>178</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>179</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>180</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>181</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>182</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>183</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>184</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>185</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>186</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>187</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>188</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>189</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>190</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>191</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>192</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>193</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>194</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>195</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>196</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>197</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>198</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>199</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>200</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>201</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>202</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:71" x14ac:dyDescent="0.25">
@@ -29887,211 +29887,211 @@
         <v>134</v>
       </c>
       <c r="C1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>137</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>139</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>140</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>141</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>142</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>143</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>144</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>145</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>146</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>147</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>148</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>149</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>150</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>151</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>152</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>153</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>154</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>155</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>156</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>157</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>158</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>159</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>160</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>161</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>162</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>163</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>164</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>165</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>166</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>167</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>168</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>169</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>170</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>171</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>172</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>173</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>174</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>175</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>176</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>177</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>178</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>179</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>180</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>181</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>182</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>183</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>184</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>185</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>186</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>187</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>188</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>189</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>190</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>191</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>192</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>193</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BK1" t="s">
         <v>194</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>195</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" t="s">
         <v>196</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
         <v>197</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BO1" t="s">
         <v>198</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BP1" t="s">
         <v>199</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>200</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>201</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
         <v>202</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:71" x14ac:dyDescent="0.25">
@@ -32438,15 +32438,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001E2F74E811AAA4409A164A292B7ABC74" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a274884ad72c80bb9b486423286f1f97">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="728ae82c-3d1b-45f0-8d67-959bce25b5b0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0920719d7b65f5660acd9896835e0dd0" ns3:_="">
     <xsd:import namespace="728ae82c-3d1b-45f0-8d67-959bce25b5b0"/>
@@ -32596,6 +32587,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9EAE9DF-01E1-49E5-8603-E69C76183A40}">
   <ds:schemaRefs>
@@ -32613,14 +32613,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FABF7966-B5A2-43B3-86A8-0DA6CE927C7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45043DEE-C555-410D-B3FE-BB9490E0CF46}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32636,4 +32628,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FABF7966-B5A2-43B3-86A8-0DA6CE927C7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>